<commit_message>
Templates: remove case-study branding, credit Olugboye Shola
All 15 templates (md, csv, docx, xlsx) are now unbranded: no scenario names,
project IDs or case-study notices. Each carries one credit line.

Claude-Session: https://claude.ai/code/session_0165XZisJZG4P3mrG9rbChTW
</commit_message>
<xml_diff>
--- a/templates/iso27001-soa-template.xlsx
+++ b/templates/iso27001-soa-template.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">ISO/IEC 27001:2022 Statement of Applicability &amp; Readiness - Template</t>
   </si>
   <si>
-    <t xml:space="preserve">TEMPLATE - replace every blank yellow cell. Derived from the simulated CGI-ISO-001 portfolio project. ISO/IEC 27001 wording is paraphrased; use the purchased standard.</t>
+    <t xml:space="preserve">TEMPLATE - replace every blank yellow cell. Prepared by Olugboye Shola. ISO/IEC 27001 wording is paraphrased; use the purchased standard.</t>
   </si>
   <si>
     <t xml:space="preserve">What it does</t>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">If any gate requirement (4.3, 6.1.2, 6.1.3, 9.2.1, 9.2.2, 9.3.1, 9.3.2, 9.3.3) scores below 2, the Stage 1 decision is NO-GO whatever the percentage.</t>
   </si>
   <si>
-    <t xml:space="preserve">Worked example (simulated)</t>
+    <t xml:space="preserve">Worked example</t>
   </si>
   <si>
     <t xml:space="preserve">A.8.13 Information backup | Y | Acts after the event to limit the impact of ransomware; snapshots exist but no restore has been tested, so no credit is taken | maturity 1 -&gt; Partial | Held: backup configuration. Required: backup policy; dated restore test | IT Operations Manager | R-002 | PR.IR; RC.RP | F-013</t>

</xml_diff>